<commit_message>
docs: record completed notation phase 3 acceptance
</commit_message>
<xml_diff>
--- a/docs/evolution/roadmap-notation.xlsx
+++ b/docs/evolution/roadmap-notation.xlsx
@@ -820,7 +820,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1095,13 +1095,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>51 assertions executed; §4 of harness-notation.md</t>
+          <t>53 assertions executed; §4 of harness-notation.md</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Say what the surface is, and make the oracles part of the toolchain: `oracles` dev extra, vendored XSD, fixture corpus, runner, ADR-0009, proof-sheet labelling, interim tuning diagnostic</t>
+          <t>Say what the surface is, and make the oracles part of the toolchain: `oracles` dev extra, vendored XSD, fixture corpus, runner, ADR-0011, proof-sheet labelling, interim tuning diagnostic</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -1499,13 +1499,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1837,15 +1837,17 @@
       </c>
       <c r="Z2" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA2" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB2" s="4" t="inlineStr">
         <is>
-          <t>README diff</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NDOC-003</t>
         </is>
       </c>
       <c r="AC2" s="4" t="inlineStr">
@@ -1993,15 +1995,17 @@
       </c>
       <c r="Z3" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA3" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA3" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB3" s="4" t="inlineStr">
         <is>
-          <t>doc diff</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NDOC-004</t>
         </is>
       </c>
       <c r="AC3" s="4" t="inlineStr">
@@ -2048,7 +2052,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009: notation positioning — semantic score contract + oracle-verified interchange; engraving and deep musicology delegated to LilyPond and music21; proof sheet retained</t>
+          <t>ADR-0011: notation positioning — semantic score contract + oracle-verified interchange; engraving and deep musicology delegated to LilyPond and music21; proof sheet retained</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
@@ -2149,15 +2153,17 @@
       </c>
       <c r="Z4" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA4" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>docs/adr/0009-*.md</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NDOC-005</t>
         </is>
       </c>
       <c r="AC4" s="4" t="inlineStr">
@@ -2305,15 +2311,17 @@
       </c>
       <c r="Z5" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA5" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA5" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>docs/backlog.yml</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NGATE-006</t>
         </is>
       </c>
       <c r="AC5" s="4" t="inlineStr">
@@ -2465,15 +2473,17 @@
       </c>
       <c r="Z6" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA6" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA6" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>pyproject diff; tests/fixtures/musicxml/xsd/</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NORA-001, HARNESS-NORA-002</t>
         </is>
       </c>
       <c r="AC6" s="4" t="inlineStr">
@@ -2625,15 +2635,17 @@
       </c>
       <c r="Z7" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA7" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA7" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>tests/fixtures/notation/</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NGATE-001</t>
         </is>
       </c>
       <c r="AC7" s="4" t="inlineStr">
@@ -2785,15 +2797,17 @@
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA8" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>pytest log with the extra</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NORA-003, HARNESS-NXML-001, HARNESS-NXML-010, HARNESS-NENG-001, HARNESS-NANA-001, HARNESS-NGATE-002, HARNESS-NGATE-003, HARNESS-NGATE-004, HARNESS-NANA-003, HARNESS-NMIDI-001</t>
         </is>
       </c>
       <c r="AC8" s="4" t="inlineStr"/>
@@ -2926,7 +2940,7 @@
       </c>
       <c r="W9" s="4" t="inlineStr">
         <is>
-          <t>`scripts/harness-notation.sh T1` produces summary.tsv with all 51 IDs</t>
+          <t>`scripts/harness-notation.sh T1` produces summary.tsv with all 53 IDs</t>
         </is>
       </c>
       <c r="X9" s="4" t="inlineStr">
@@ -2941,15 +2955,17 @@
       </c>
       <c r="Z9" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA9" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA9" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>evidence-notation/T1/summary.tsv</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NGATE-005</t>
         </is>
       </c>
       <c r="AC9" s="4" t="inlineStr">
@@ -3101,15 +3117,17 @@
       </c>
       <c r="Z10" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA10" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA10" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>docs diff</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NENG-003</t>
         </is>
       </c>
       <c r="AC10" s="4" t="inlineStr">
@@ -3261,15 +3279,17 @@
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA11" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA11" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>diagnostic in compile output</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NTUN-003</t>
         </is>
       </c>
       <c r="AC11" s="4" t="inlineStr">
@@ -3421,15 +3441,17 @@
       </c>
       <c r="Z12" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA12" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA12" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
-          <t>import of vendored chorale</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NIMP-001</t>
         </is>
       </c>
       <c r="AC12" s="4" t="inlineStr"/>
@@ -3577,15 +3599,17 @@
       </c>
       <c r="Z13" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA13" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA13" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
-          <t>import tests</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NIMP-002</t>
         </is>
       </c>
       <c r="AC13" s="4" t="inlineStr"/>
@@ -3729,15 +3753,17 @@
       </c>
       <c r="Z14" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA14" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA14" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
-          <t>import tests</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NIMP-003</t>
         </is>
       </c>
       <c r="AC14" s="4" t="inlineStr"/>
@@ -3885,15 +3911,17 @@
       </c>
       <c r="Z15" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA15" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA15" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB15" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-002</t>
         </is>
       </c>
       <c r="AC15" s="4" t="inlineStr"/>
@@ -4041,15 +4069,17 @@
       </c>
       <c r="Z16" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA16" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA16" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB16" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-003</t>
         </is>
       </c>
       <c r="AC16" s="4" t="inlineStr"/>
@@ -4197,15 +4227,17 @@
       </c>
       <c r="Z17" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA17" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA17" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB17" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-004</t>
         </is>
       </c>
       <c r="AC17" s="4" t="inlineStr"/>
@@ -4353,15 +4385,17 @@
       </c>
       <c r="Z18" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA18" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA18" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB18" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-005</t>
         </is>
       </c>
       <c r="AC18" s="4" t="inlineStr"/>
@@ -4509,15 +4543,17 @@
       </c>
       <c r="Z19" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA19" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA19" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB19" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-009, HARNESS-NMIDI-002, HARNESS-NMIDI-003</t>
         </is>
       </c>
       <c r="AC19" s="4" t="inlineStr"/>
@@ -4665,15 +4701,17 @@
       </c>
       <c r="Z20" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA20" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA20" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB20" s="4" t="inlineStr">
         <is>
-          <t>tests/test_notation_oracles.py</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NANA-001, HARNESS-NANA-002</t>
         </is>
       </c>
       <c r="AC20" s="4" t="inlineStr"/>
@@ -4821,15 +4859,17 @@
       </c>
       <c r="Z21" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA21" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA21" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB21" s="4" t="inlineStr">
         <is>
-          <t>generated manifest</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NDOC-002</t>
         </is>
       </c>
       <c r="AC21" s="4" t="inlineStr"/>
@@ -4973,15 +5013,17 @@
       </c>
       <c r="Z22" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA22" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA22" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB22" s="4" t="inlineStr">
         <is>
-          <t>tests/fixtures/notation/corpus/</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NIMP-004</t>
         </is>
       </c>
       <c r="AC22" s="4" t="inlineStr"/>
@@ -5125,15 +5167,17 @@
       </c>
       <c r="Z23" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA23" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA23" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB23" s="4" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NIMP-005</t>
         </is>
       </c>
       <c r="AC23" s="4" t="inlineStr"/>
@@ -5281,15 +5325,17 @@
       </c>
       <c r="Z24" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA24" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA24" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB24" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-006</t>
         </is>
       </c>
       <c r="AC24" s="4" t="inlineStr"/>
@@ -5437,15 +5483,17 @@
       </c>
       <c r="Z25" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA25" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA25" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB25" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-007</t>
         </is>
       </c>
       <c r="AC25" s="4" t="inlineStr"/>
@@ -5589,15 +5637,17 @@
       </c>
       <c r="Z26" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA26" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA26" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB26" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-008</t>
         </is>
       </c>
       <c r="AC26" s="4" t="inlineStr"/>
@@ -5745,15 +5795,17 @@
       </c>
       <c r="Z27" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA27" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA27" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB27" s="4" t="inlineStr">
         <is>
-          <t>fixture exports</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NSEM-002</t>
         </is>
       </c>
       <c r="AC27" s="4" t="inlineStr"/>
@@ -5901,15 +5953,17 @@
       </c>
       <c r="Z28" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA28" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA28" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
-          <t>docs/INTEROP.md generated section</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NXML-011, HARNESS-NSEM-001, HARNESS-NDOC-001</t>
         </is>
       </c>
       <c r="AC28" s="4" t="inlineStr"/>
@@ -7067,7 +7121,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009 records the decision</t>
+          <t>ADR-0011 records the decision</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -7157,15 +7211,17 @@
       </c>
       <c r="Z36" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
-        </is>
-      </c>
-      <c r="AA36" s="4" t="n">
-        <v>0</v>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="AA36" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="AB36" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009</t>
+          <t>docs/evolution/evidence-notation/T3/results.json; HARNESS-NANA-005</t>
         </is>
       </c>
       <c r="AC36" s="4" t="inlineStr"/>
@@ -7348,13 +7404,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -8353,7 +8409,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009: notation positioning — semantic score contract + o</t>
+          <t>ADR-0011: notation positioning — semantic score contract + o</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -8449,7 +8505,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009: notation positioning — semantic score contract + o</t>
+          <t>ADR-0011: notation positioning — semantic score contract + o</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -8525,13 +8581,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -8619,7 +8675,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>51 assertions executed; §4 of harness-notation.md</t>
+          <t>53 assertions executed; §4 of harness-notation.md</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -8651,7 +8707,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Say what the surface is, and make the oracles part of the toolchain: `oracles` dev extra, vendored XSD, fixture corpus, runner, ADR-0009, proof-sheet labelling, interim tuning diagnostic</t>
+          <t>Say what the surface is, and make the oracles part of the toolchain: `oracles` dev extra, vendored XSD, fixture corpus, runner, ADR-0011, proof-sheet labelling, interim tuning diagnostic</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -8671,7 +8727,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -8713,7 +8769,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8811,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>not-started</t>
+          <t>complete (T3 evidence)</t>
         </is>
       </c>
     </row>
@@ -8888,13 +8944,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -10853,7 +10909,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>ADR-0009 records the positioning: semantic score contract, oracle-verified interchange, engraving and musicology delegated, proof sheet retained</t>
+          <t>ADR-0011 records the positioning: semantic score contract, oracle-verified interchange, engraving and musicology delegated, proof sheet retained</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -11454,13 +11510,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -12069,13 +12125,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -12363,13 +12419,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -12600,7 +12656,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>parity test; ADR-0009</t>
+          <t>parity test; ADR-0011</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -12740,7 +12796,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>